<commit_message>
se tiene el codigo funcional con los remark
</commit_message>
<xml_diff>
--- a/PlanStaffRGM.xlsx
+++ b/PlanStaffRGM.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Operations_best_opt" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operations_best_opt" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -56328,6 +56328,41 @@
           <t>T</t>
         </is>
       </c>
+      <c r="ATF14" s="109" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ATG14" s="109" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ATH14" s="109" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ATI14" s="109" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ATJ14" s="109" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ATK14" s="109" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ATL14" s="109" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="9">

</xml_diff>

<commit_message>
se hace modificacion para solucionar el problema de merge en la BD, queda pendiente hacer test total. Despues de la fase de test se hace push
</commit_message>
<xml_diff>
--- a/PlanStaffRGM.xlsx
+++ b/PlanStaffRGM.xlsx
@@ -1344,7 +1344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AWU14"/>
+  <dimension ref="A1:AWU16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -56461,6 +56461,40 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Supervisor</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Camilo Zapata</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>BNM321</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Supervisor</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Camilo Zapata</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>BNM159</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="YT7:YX7"/>

</xml_diff>

<commit_message>
se tiene los datos del reporte inbound outbound con respecto a la informacion de entry y out date
</commit_message>
<xml_diff>
--- a/PlanStaffRGM.xlsx
+++ b/PlanStaffRGM.xlsx
@@ -48360,6 +48360,36 @@
           <t>ON NS</t>
         </is>
       </c>
+      <c r="AUA13" s="109" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AUB13" s="109" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AUC13" s="109" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AUD13" s="109" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AUE13" s="109" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AUF13" s="109" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -48570,6 +48600,36 @@
       <c r="ATY14" s="109" t="inlineStr">
         <is>
           <t>ON</t>
+        </is>
+      </c>
+      <c r="AUA14" s="111" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="AUB14" s="111" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="AUC14" s="111" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="AUD14" s="111" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="AUE14" s="111" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="AUF14" s="111" t="inlineStr">
+        <is>
+          <t>ON NS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Funciona la generacion de reporte con entry date y exit date
</commit_message>
<xml_diff>
--- a/PlanStaffRGM.xlsx
+++ b/PlanStaffRGM.xlsx
@@ -989,6 +989,36 @@
       <text>
         <t>Data Analyst:
 will take in July as compensation leave</t>
+      </text>
+    </comment>
+    <comment ref="AUA12" authorId="1" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AUB12" authorId="1" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AUC12" authorId="1" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AUD12" authorId="1" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AUE12" authorId="1" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AUF12" authorId="1" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
       </text>
     </comment>
     <comment ref="ASN14" authorId="1" shapeId="0">
@@ -48308,6 +48338,36 @@
           <t>ON</t>
         </is>
       </c>
+      <c r="AUA12" s="113" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AUB12" s="113" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AUC12" s="113" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AUD12" s="113" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AUE12" s="113" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AUF12" s="113" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">

</xml_diff>

<commit_message>
se cumple el requeriiento de la carga en funcion de la maquina y procesos y no en funcion de un delay
</commit_message>
<xml_diff>
--- a/PlanStaffRGM.xlsx
+++ b/PlanStaffRGM.xlsx
@@ -73,7 +73,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -144,6 +144,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC7CE"/>
         <bgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -240,7 +246,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -414,6 +420,7 @@
     <xf numFmtId="46" fontId="5" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>

</xml_diff>

<commit_message>
Se registran los datos haciendo el scroll right
</commit_message>
<xml_diff>
--- a/PlanStaffRGM.xlsx
+++ b/PlanStaffRGM.xlsx
@@ -73,7 +73,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -150,6 +150,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
         <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF99"/>
+        <bgColor rgb="00FFFF99"/>
       </patternFill>
     </fill>
   </fills>
@@ -246,7 +258,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -424,6 +436,11 @@
     <xf numFmtId="164" fontId="4" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -10840,11 +10857,31 @@
       </c>
       <c r="AVS2" s="12" t="n"/>
       <c r="AVT2" s="12" t="n"/>
-      <c r="AVU2" s="12" t="n"/>
-      <c r="AVV2" s="12" t="n"/>
-      <c r="AVW2" s="12" t="n"/>
-      <c r="AVX2" s="12" t="n"/>
-      <c r="AVY2" s="12" t="n"/>
+      <c r="AVU2" s="63" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AVV2" s="63" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AVW2" s="63" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AVX2" s="63" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AVY2" s="63" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
       <c r="AVZ2" s="12" t="n"/>
       <c r="AWA2" s="12" t="n"/>
       <c r="AWB2" s="12" t="n"/>
@@ -35549,11 +35586,7 @@
       </c>
     </row>
     <row r="8" ht="30" customFormat="1" customHeight="1" s="8">
-      <c r="A8" s="13" t="inlineStr">
-        <is>
-          <t>Technician</t>
-        </is>
-      </c>
+      <c r="A8" s="13" t="inlineStr"/>
       <c r="B8" s="14" t="inlineStr">
         <is>
           <t>Clemente Nufable</t>
@@ -39805,6 +39838,41 @@
         </is>
       </c>
       <c r="ASW8" s="27" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AVU8" s="64" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AVV8" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AVW8" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AVX8" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AVY8" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AVZ8" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AWA8" s="61" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
@@ -46321,7 +46389,6 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
           <t>Rosa Melano</t>

</xml_diff>

<commit_message>
se agrega la opcion de Travel date are different from work Period en el dropdown del preview schedule para que se asigne la info al  hacer scroll right
</commit_message>
<xml_diff>
--- a/PlanStaffRGM.xlsx
+++ b/PlanStaffRGM.xlsx
@@ -16735,11 +16735,7 @@
       </c>
     </row>
     <row r="4" ht="30" customFormat="1" customHeight="1" s="8">
-      <c r="A4" s="13" t="inlineStr">
-        <is>
-          <t>Technician</t>
-        </is>
-      </c>
+      <c r="A4" s="13" t="inlineStr"/>
       <c r="B4" s="14" t="inlineStr">
         <is>
           <t>Randolf Padernal</t>
@@ -21602,6 +21598,31 @@
       <c r="ASW4" s="37" t="inlineStr">
         <is>
           <t>OFF</t>
+        </is>
+      </c>
+      <c r="AVU4" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AVV4" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AVW4" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AVX4" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AVY4" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Se realiza correccion con respecto al scroll right para los turnos creados por shift
</commit_message>
<xml_diff>
--- a/PlanStaffRGM.xlsx
+++ b/PlanStaffRGM.xlsx
@@ -73,7 +73,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -162,6 +162,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFFF99"/>
         <bgColor rgb="00FFFF99"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF0000"/>
+        <bgColor rgb="00FF0000"/>
       </patternFill>
     </fill>
   </fills>
@@ -258,7 +264,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -441,6 +447,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -521,119 +528,124 @@
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
+    <author>ShiftType</author>
     <author>Data Analyst</author>
-    <author>ShiftType</author>
   </authors>
   <commentList>
-    <comment ref="ALX9" authorId="0" shapeId="0">
+    <comment ref="AWB4" authorId="0" shapeId="0">
+      <text>
+        <t>08:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="ALX9" authorId="1" shapeId="0">
       <text>
         <t>Data Analyst:
 will take in July as compensation leave</t>
       </text>
     </comment>
-    <comment ref="ALY9" authorId="0" shapeId="0">
+    <comment ref="ALY9" authorId="1" shapeId="0">
       <text>
         <t>Data Analyst:
 will take in July as compensation leave</t>
       </text>
     </comment>
-    <comment ref="ALZ9" authorId="0" shapeId="0">
+    <comment ref="ALZ9" authorId="1" shapeId="0">
       <text>
         <t>Data Analyst:
 will take in July as compensation leave</t>
       </text>
     </comment>
-    <comment ref="AUA11" authorId="1" shapeId="0">
+    <comment ref="AUA11" authorId="0" shapeId="0">
       <text>
         <t>13:00-17:00</t>
       </text>
     </comment>
-    <comment ref="AUB11" authorId="1" shapeId="0">
+    <comment ref="AUB11" authorId="0" shapeId="0">
       <text>
         <t>13:00-17:00</t>
       </text>
     </comment>
-    <comment ref="AUC11" authorId="1" shapeId="0">
+    <comment ref="AUC11" authorId="0" shapeId="0">
       <text>
         <t>13:00-17:00</t>
       </text>
     </comment>
-    <comment ref="AUD11" authorId="1" shapeId="0">
+    <comment ref="AUD11" authorId="0" shapeId="0">
       <text>
         <t>13:00-17:00</t>
       </text>
     </comment>
-    <comment ref="AUE11" authorId="1" shapeId="0">
+    <comment ref="AUE11" authorId="0" shapeId="0">
       <text>
         <t>13:00-17:00</t>
       </text>
     </comment>
-    <comment ref="AUF11" authorId="1" shapeId="0">
+    <comment ref="AUF11" authorId="0" shapeId="0">
       <text>
         <t>13:00-17:00</t>
       </text>
     </comment>
-    <comment ref="ASN13" authorId="1" shapeId="0">
+    <comment ref="ASN13" authorId="0" shapeId="0">
       <text>
         <t>08:00-17:00</t>
       </text>
     </comment>
-    <comment ref="ASO13" authorId="1" shapeId="0">
+    <comment ref="ASO13" authorId="0" shapeId="0">
       <text>
         <t>08:00-17:00</t>
       </text>
     </comment>
-    <comment ref="ASP13" authorId="1" shapeId="0">
+    <comment ref="ASP13" authorId="0" shapeId="0">
       <text>
         <t>08:00-17:00</t>
       </text>
     </comment>
-    <comment ref="ASQ13" authorId="1" shapeId="0">
+    <comment ref="ASQ13" authorId="0" shapeId="0">
       <text>
         <t>08:00-17:00</t>
       </text>
     </comment>
-    <comment ref="ASR13" authorId="1" shapeId="0">
+    <comment ref="ASR13" authorId="0" shapeId="0">
       <text>
         <t>08:00-17:00</t>
       </text>
     </comment>
-    <comment ref="ASU13" authorId="1" shapeId="0">
+    <comment ref="ASU13" authorId="0" shapeId="0">
       <text>
         <t>08:00-17:00</t>
       </text>
     </comment>
-    <comment ref="ASV13" authorId="1" shapeId="0">
+    <comment ref="ASV13" authorId="0" shapeId="0">
       <text>
         <t>08:00-17:00</t>
       </text>
     </comment>
-    <comment ref="ASW13" authorId="1" shapeId="0">
+    <comment ref="ASW13" authorId="0" shapeId="0">
       <text>
         <t>08:00-17:00</t>
       </text>
     </comment>
-    <comment ref="ASX13" authorId="1" shapeId="0">
+    <comment ref="ASX13" authorId="0" shapeId="0">
       <text>
         <t>08:00-17:00</t>
       </text>
     </comment>
-    <comment ref="ATB13" authorId="1" shapeId="0">
+    <comment ref="ATB13" authorId="0" shapeId="0">
       <text>
         <t>13:00-17:00</t>
       </text>
     </comment>
-    <comment ref="ATC13" authorId="1" shapeId="0">
+    <comment ref="ATC13" authorId="0" shapeId="0">
       <text>
         <t>13:00-17:00</t>
       </text>
     </comment>
-    <comment ref="ATD13" authorId="1" shapeId="0">
+    <comment ref="ATD13" authorId="0" shapeId="0">
       <text>
         <t>13:00-17:00</t>
       </text>
     </comment>
-    <comment ref="ATE13" authorId="1" shapeId="0">
+    <comment ref="ATE13" authorId="0" shapeId="0">
       <text>
         <t>13:00-17:00</t>
       </text>
@@ -10884,12 +10896,36 @@
       </c>
       <c r="AVZ2" s="12" t="n"/>
       <c r="AWA2" s="12" t="n"/>
-      <c r="AWB2" s="12" t="n"/>
-      <c r="AWC2" s="12" t="n"/>
-      <c r="AWD2" s="12" t="n"/>
-      <c r="AWE2" s="12" t="n"/>
-      <c r="AWF2" s="12" t="n"/>
-      <c r="AWG2" s="12" t="n"/>
+      <c r="AWB2" s="62" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AWC2" s="62" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AWD2" s="62" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AWE2" s="62" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AWF2" s="62" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AWG2" s="62" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
       <c r="AWH2" s="12" t="n"/>
       <c r="AWI2" s="12" t="n"/>
       <c r="AWJ2" s="12" t="n"/>
@@ -21623,6 +21659,36 @@
       <c r="AVY4" s="61" t="inlineStr">
         <is>
           <t>ON</t>
+        </is>
+      </c>
+      <c r="AWB4" s="66" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="AWC4" s="66" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="AWD4" s="66" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="AWE4" s="66" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="AWF4" s="66" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="AWG4" s="66" t="inlineStr">
+        <is>
+          <t>S</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
el time del primero en seleccionar por dropdown respalda a los que se hacen por scroll right
</commit_message>
<xml_diff>
--- a/PlanStaffRGM.xlsx
+++ b/PlanStaffRGM.xlsx
@@ -73,7 +73,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -170,6 +170,12 @@
         <bgColor rgb="00FF0000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC000"/>
+        <bgColor rgb="00FFC000"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="7">
     <border>
@@ -264,7 +270,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -448,6 +454,7 @@
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -532,7 +539,67 @@
     <author>Data Analyst</author>
   </authors>
   <commentList>
+    <comment ref="AWB3" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AWC3" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AWD3" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AWE3" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AWF3" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AWG3" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
     <comment ref="AWB4" authorId="0" shapeId="0">
+      <text>
+        <t>08:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AWB6" authorId="0" shapeId="0">
+      <text>
+        <t>08:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AWC6" authorId="0" shapeId="0">
+      <text>
+        <t>08:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AWD6" authorId="0" shapeId="0">
+      <text>
+        <t>08:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AWE6" authorId="0" shapeId="0">
+      <text>
+        <t>08:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AWF6" authorId="0" shapeId="0">
+      <text>
+        <t>08:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AWG6" authorId="0" shapeId="0">
       <text>
         <t>08:00-17:00</t>
       </text>
@@ -10942,11 +11009,7 @@
       <c r="AWU2" s="12" t="n"/>
     </row>
     <row r="3" ht="30" customFormat="1" customHeight="1" s="8">
-      <c r="A3" s="13" t="inlineStr">
-        <is>
-          <t>Technician</t>
-        </is>
-      </c>
+      <c r="A3" s="13" t="inlineStr"/>
       <c r="B3" s="14" t="inlineStr">
         <is>
           <t>Romeo Bean</t>
@@ -16767,6 +16830,36 @@
       <c r="ASY3" s="26" t="inlineStr">
         <is>
           <t>ON</t>
+        </is>
+      </c>
+      <c r="AWB3" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AWC3" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AWD3" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AWE3" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AWF3" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AWG3" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -26808,11 +26901,7 @@
       </c>
     </row>
     <row r="6" ht="30" customFormat="1" customHeight="1" s="8">
-      <c r="A6" s="13" t="inlineStr">
-        <is>
-          <t>Technician</t>
-        </is>
-      </c>
+      <c r="A6" s="13" t="inlineStr"/>
       <c r="B6" s="14" t="inlineStr">
         <is>
           <t>Jean Atmidi</t>
@@ -31283,6 +31372,36 @@
       <c r="ASW6" s="27" t="inlineStr">
         <is>
           <t>ON</t>
+        </is>
+      </c>
+      <c r="AWB6" s="66" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="AWC6" s="66" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="AWD6" s="66" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="AWE6" s="66" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="AWF6" s="66" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="AWG6" s="66" t="inlineStr">
+        <is>
+          <t>S</t>
         </is>
       </c>
     </row>
@@ -39966,11 +40085,7 @@
       </c>
     </row>
     <row r="9" ht="30" customFormat="1" customHeight="1" s="8">
-      <c r="A9" s="13" t="inlineStr">
-        <is>
-          <t>Technician</t>
-        </is>
-      </c>
+      <c r="A9" s="13" t="inlineStr"/>
       <c r="B9" s="14" t="inlineStr">
         <is>
           <t>Akshay Mangroe</t>
@@ -44816,6 +44931,11 @@
         </is>
       </c>
       <c r="ATE9" s="26" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AWB9" s="61" t="inlineStr">
         <is>
           <t>ON</t>
         </is>

</xml_diff>

<commit_message>
Los scrolls right toman la hora entry y exit
</commit_message>
<xml_diff>
--- a/PlanStaffRGM.xlsx
+++ b/PlanStaffRGM.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Operations_best_opt" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operations_best_opt" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -46397,11 +46397,7 @@
       </c>
     </row>
     <row r="11" ht="30" customFormat="1" customHeight="1" s="8">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Supervisor</t>
-        </is>
-      </c>
+      <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
           <t>Elver Gonzales</t>
@@ -46510,6 +46506,76 @@
       <c r="AUF11" s="30" t="inlineStr">
         <is>
           <t>T</t>
+        </is>
+      </c>
+      <c r="AVR11" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AVS11" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AVT11" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AVU11" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AVV11" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AWB11" s="65" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="AWC11" s="65" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="AWD11" s="65" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="AWE11" s="65" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="AWG11" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AWH11" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AWI11" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AWJ11" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AWK11" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
intervalo entre PeriodStartDate and PeriodEndDate
</commit_message>
<xml_diff>
--- a/PlanStaffRGM.xlsx
+++ b/PlanStaffRGM.xlsx
@@ -574,6 +574,41 @@
         <t>08:00-17:00</t>
       </text>
     </comment>
+    <comment ref="AVU6" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AVV6" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AVW6" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AVX6" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AVY6" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AVZ6" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AWA6" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
     <comment ref="AWB6" authorId="0" shapeId="0">
       <text>
         <t>08:00-17:00</t>
@@ -602,6 +637,106 @@
     <comment ref="AWG6" authorId="0" shapeId="0">
       <text>
         <t>08:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AVM7" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AVN7" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AVO7" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AVP7" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AVQ7" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AVR7" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AVU7" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AVV7" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AVW7" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AVX7" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AVY7" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AVZ7" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AWA7" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AWM7" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AWN7" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AWO7" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AWP7" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AWQ7" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AWR7" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="AWS7" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
       </text>
     </comment>
     <comment ref="ALX9" authorId="1" shapeId="0">
@@ -10998,14 +11133,46 @@
       <c r="AWJ2" s="12" t="n"/>
       <c r="AWK2" s="12" t="n"/>
       <c r="AWL2" s="12" t="n"/>
-      <c r="AWM2" s="12" t="n"/>
-      <c r="AWN2" s="12" t="n"/>
-      <c r="AWO2" s="12" t="n"/>
-      <c r="AWP2" s="12" t="n"/>
-      <c r="AWQ2" s="12" t="n"/>
-      <c r="AWR2" s="12" t="n"/>
-      <c r="AWS2" s="12" t="n"/>
-      <c r="AWT2" s="12" t="n"/>
+      <c r="AWM2" s="63" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AWN2" s="63" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AWO2" s="63" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AWP2" s="63" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AWQ2" s="63" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AWR2" s="63" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AWS2" s="63" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AWT2" s="63" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
       <c r="AWU2" s="12" t="n"/>
     </row>
     <row r="3" ht="30" customFormat="1" customHeight="1" s="8">
@@ -21782,6 +21949,41 @@
       <c r="AWG4" s="66" t="inlineStr">
         <is>
           <t>S</t>
+        </is>
+      </c>
+      <c r="AWM4" s="65" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="AWN4" s="65" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="AWO4" s="65" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="AWP4" s="65" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="AWQ4" s="65" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="AWR4" s="65" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="AWS4" s="65" t="inlineStr">
+        <is>
+          <t>ON NS</t>
         </is>
       </c>
     </row>
@@ -31374,6 +31576,41 @@
           <t>ON</t>
         </is>
       </c>
+      <c r="AVU6" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AVV6" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AVW6" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AVX6" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AVY6" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AVZ6" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AWA6" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
       <c r="AWB6" s="66" t="inlineStr">
         <is>
           <t>S</t>
@@ -31406,11 +31643,7 @@
       </c>
     </row>
     <row r="7" ht="30" customFormat="1" customHeight="1" s="8">
-      <c r="A7" s="13" t="inlineStr">
-        <is>
-          <t>Technician</t>
-        </is>
-      </c>
+      <c r="A7" s="13" t="inlineStr"/>
       <c r="B7" s="14" t="inlineStr">
         <is>
           <t>Manuel Corral</t>
@@ -35788,6 +36021,106 @@
       <c r="ASW7" s="27" t="inlineStr">
         <is>
           <t>ON</t>
+        </is>
+      </c>
+      <c r="AVM7" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AVN7" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AVO7" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AVP7" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AVQ7" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AVR7" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AVU7" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AVV7" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AVW7" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AVX7" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AVY7" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AVZ7" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AWA7" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AWM7" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AWN7" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AWO7" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AWP7" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AWQ7" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AWR7" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="AWS7" s="67" t="inlineStr">
+        <is>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -40048,9 +40381,9 @@
           <t>ON</t>
         </is>
       </c>
-      <c r="AVU8" s="64" t="inlineStr">
-        <is>
-          <t>OFF</t>
+      <c r="AVU8" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
         </is>
       </c>
       <c r="AVV8" s="61" t="inlineStr">
@@ -44933,6 +45266,41 @@
       <c r="ATE9" s="26" t="inlineStr">
         <is>
           <t>ON</t>
+        </is>
+      </c>
+      <c r="AVU9" s="65" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="AVV9" s="65" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="AVW9" s="65" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="AVX9" s="65" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="AVY9" s="65" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="AVZ9" s="65" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="AWA9" s="65" t="inlineStr">
+        <is>
+          <t>ON NS</t>
         </is>
       </c>
       <c r="AWB9" s="61" t="inlineStr">
@@ -46397,7 +46765,6 @@
       </c>
     </row>
     <row r="11" ht="30" customFormat="1" customHeight="1" s="8">
-      <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
           <t>Elver Gonzales</t>
@@ -46580,11 +46947,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Site Manager</t>
-        </is>
-      </c>
+      <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
           <t>Miguel Venegas</t>
@@ -46656,6 +47019,26 @@
         </is>
       </c>
       <c r="AUF12" s="26" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AWR12" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AWS12" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AWT12" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AWU12" s="61" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
@@ -46900,6 +47283,91 @@
       <c r="AVR13" s="61" t="inlineStr">
         <is>
           <t>ON</t>
+        </is>
+      </c>
+      <c r="AVV13" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AVW13" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AVX13" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AVY13" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AVZ13" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AWB13" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AWC13" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AWD13" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AWE13" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AWF13" s="61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AWM13" s="64" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AWN13" s="64" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AWO13" s="64" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AWP13" s="64" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AWQ13" s="64" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AWR13" s="64" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AWS13" s="64" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
edit day schedule bug solucionado
</commit_message>
<xml_diff>
--- a/PlanStaffRGM.xlsx
+++ b/PlanStaffRGM.xlsx
@@ -27,7 +27,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -52,6 +52,12 @@
         <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC000"/>
+        <bgColor rgb="00FFC000"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -65,12 +71,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -145,6 +152,41 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>ShiftType</author>
+  </authors>
+  <commentList>
+    <comment ref="S2" authorId="0" shapeId="0">
+      <text>
+        <t>08:00-10:00</t>
+      </text>
+    </comment>
+    <comment ref="T2" authorId="0" shapeId="0">
+      <text>
+        <t>08:00-10:00</t>
+      </text>
+    </comment>
+    <comment ref="U2" authorId="0" shapeId="0">
+      <text>
+        <t>08:00-10:00</t>
+      </text>
+    </comment>
+    <comment ref="V2" authorId="0" shapeId="0">
+      <text>
+        <t>08:00-10:00</t>
+      </text>
+    </comment>
+    <comment ref="W2" authorId="0" shapeId="0">
+      <text>
+        <t>08:00-10:00</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -782,6 +824,36 @@
           <t>OFF</t>
         </is>
       </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="S2" s="5" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="T2" s="5" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="U2" s="5" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="V2" s="5" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="W2" s="5" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="B3" t="inlineStr">
@@ -839,6 +911,31 @@
           <t>ON NS</t>
         </is>
       </c>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="W3" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="B4" t="inlineStr">
@@ -906,8 +1003,29 @@
           <t>ON</t>
         </is>
       </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="S4" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="T4" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
solucion de conflicto de cierra de ventana Edit Day Schedule solucionado antes tenia que cerrar la ventana dos veces actualmente con solo cierre desaparece la ventana
</commit_message>
<xml_diff>
--- a/PlanStaffRGM.xlsx
+++ b/PlanStaffRGM.xlsx
@@ -854,6 +854,26 @@
           <t>R</t>
         </is>
       </c>
+      <c r="Y2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="Z2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AA2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AB2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="B3" t="inlineStr">

</xml_diff>

<commit_message>
Inicializando rama DevFour con el estado actual
</commit_message>
<xml_diff>
--- a/PlanStaffRGM.xlsx
+++ b/PlanStaffRGM.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CP2"/>
+  <dimension ref="A1:CP3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="17" bestFit="1" customWidth="1" min="5" max="5"/>
@@ -835,6 +835,63 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Fuel Attendant</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Luis Hernandez</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>K159</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="S3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="T3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="U3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="V3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Arreglos solicitados despues de la version Presentado a Javier
</commit_message>
<xml_diff>
--- a/PlanStaffRGM.xlsx
+++ b/PlanStaffRGM.xlsx
@@ -27,7 +27,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -46,6 +46,24 @@
         <bgColor rgb="00FFFF99"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000055FF"/>
+        <bgColor rgb="000055FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00AA5500"/>
+        <bgColor rgb="00AA5500"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -59,12 +77,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -784,9 +805,9 @@
           <t>ON</t>
         </is>
       </c>
-      <c r="V2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
+      <c r="V2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
       <c r="W2" s="3" t="inlineStr">
@@ -807,6 +828,31 @@
       <c r="Z2" s="3" t="inlineStr">
         <is>
           <t>ON</t>
+        </is>
+      </c>
+      <c r="AA2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AB2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AC2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AD2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AE2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
       <c r="CK2" s="3" t="inlineStr">
@@ -838,55 +884,65 @@
     <row r="3">
       <c r="B3" t="inlineStr">
         <is>
-          <t>Fuel Attendant</t>
+          <t>Fuel Attentand</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Luis Hernandez</t>
+          <t>Aldair Altamirando</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>K159</t>
-        </is>
-      </c>
-      <c r="L3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="M3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="N3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="R3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="S3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="T3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="U3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="V3" s="3" t="inlineStr">
+          <t>K763</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="CK3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="CL3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="CM3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="CN3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="CO3" s="3" t="inlineStr">
         <is>
           <t>ON</t>
         </is>

</xml_diff>

<commit_message>
opcion de predefinir pick up and drop off
</commit_message>
<xml_diff>
--- a/PlanStaffRGM.xlsx
+++ b/PlanStaffRGM.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EY3"/>
+  <dimension ref="A1:EY4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="17" bestFit="1" customWidth="1" min="5" max="5"/>
@@ -1133,6 +1133,63 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Fuel Attendant</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Juan Steven</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>L159</t>
+        </is>
+      </c>
+      <c r="AG4" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AH4" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AI4" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AJ4" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AK4" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AL4" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AM4" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AN4" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Guardando cambios en improvingCopyPaste
</commit_message>
<xml_diff>
--- a/PlanStaffRGM.xlsx
+++ b/PlanStaffRGM.xlsx
@@ -939,9 +939,9 @@
           <t>L159</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -954,6 +954,26 @@
           <t>OFF</t>
         </is>
       </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
       <c r="CK2" s="3" t="inlineStr">
         <is>
           <t>ON</t>
@@ -969,19 +989,19 @@
           <t>ON</t>
         </is>
       </c>
-      <c r="CN2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="CO2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="CP2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
+      <c r="CN2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="CO2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="CP2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
       <c r="EZ2" s="3" t="inlineStr">
@@ -1006,6 +1026,51 @@
           <t>T258</t>
         </is>
       </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="CK3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="CL3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="CM3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="CN3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="CO3" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="CP3" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="B4" t="inlineStr">
@@ -1023,6 +1088,46 @@
           <t>K789</t>
         </is>
       </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
       <c r="CK4" s="3" t="inlineStr">
         <is>
           <t>ON</t>
@@ -1039,6 +1144,11 @@
         </is>
       </c>
       <c r="CN4" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="CP4" s="3" t="inlineStr">
         <is>
           <t>ON</t>
         </is>

</xml_diff>

<commit_message>
COPY PASTE Funcional Pero Requiere de Test
</commit_message>
<xml_diff>
--- a/PlanStaffRGM.xlsx
+++ b/PlanStaffRGM.xlsx
@@ -939,76 +939,6 @@
           <t>L159</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="I2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="J2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="K2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="CK2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="CL2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="CM2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="CN2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="CO2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="CP2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="EZ2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="B3" t="inlineStr">
@@ -1026,51 +956,6 @@
           <t>T258</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="CK3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="CL3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="CM3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="CN3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="CO3" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="CP3" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="B4" t="inlineStr">
@@ -1086,71 +971,6 @@
       <c r="D4" t="inlineStr">
         <is>
           <t>K789</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="L4" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="CK4" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="CL4" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="CM4" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="CN4" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="CP4" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Guardando trabajo movido desde improvingCopyPaste
</commit_message>
<xml_diff>
--- a/PlanStaffRGM.xlsx
+++ b/PlanStaffRGM.xlsx
@@ -2,22 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operations_best_opt" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -28,30 +28,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF99"/>
-        <bgColor rgb="00FFFF99"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-        <bgColor rgb="00FFC7CE"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -66,17 +48,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -439,538 +416,495 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EZ4"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9.109375" defaultRowHeight="14.4"/>
-  <cols>
-    <col width="17" bestFit="1" customWidth="1" min="5" max="5"/>
-  </cols>
+  <dimension ref="A1:ES3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>TEAM</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
           <t>ROLE</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>NAME</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>BADGE</t>
         </is>
       </c>
-      <c r="E1" s="2" t="n">
+      <c r="D1" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="E1" s="1" t="n">
+        <v>46024</v>
+      </c>
+      <c r="F1" s="1" t="n">
+        <v>46025</v>
+      </c>
+      <c r="G1" s="1" t="n">
+        <v>46026</v>
+      </c>
+      <c r="H1" s="1" t="n">
+        <v>46027</v>
+      </c>
+      <c r="I1" s="1" t="n">
+        <v>46028</v>
+      </c>
+      <c r="J1" s="1" t="n">
         <v>46029</v>
       </c>
-      <c r="F1" s="2" t="n">
+      <c r="K1" s="1" t="n">
         <v>46030</v>
       </c>
-      <c r="G1" s="2" t="n">
+      <c r="L1" s="1" t="n">
         <v>46031</v>
       </c>
-      <c r="H1" s="2" t="n">
+      <c r="M1" s="1" t="n">
         <v>46032</v>
       </c>
-      <c r="I1" s="2" t="n">
+      <c r="N1" s="1" t="n">
         <v>46033</v>
       </c>
-      <c r="J1" s="2" t="n">
-        <v>46034</v>
-      </c>
-      <c r="K1" s="2" t="n">
-        <v>46035</v>
-      </c>
-      <c r="L1" s="2" t="n">
+      <c r="O1" s="1" t="n">
         <v>46036</v>
       </c>
-      <c r="M1" s="2" t="n">
+      <c r="P1" s="1" t="n">
         <v>46037</v>
       </c>
-      <c r="N1" s="2" t="n">
+      <c r="Q1" s="1" t="n">
         <v>46038</v>
       </c>
-      <c r="O1" s="2" t="n">
-        <v>46039</v>
-      </c>
-      <c r="P1" s="2" t="n">
-        <v>46040</v>
-      </c>
-      <c r="Q1" s="2" t="n">
-        <v>46041</v>
-      </c>
-      <c r="R1" s="2" t="n">
+      <c r="R1" s="1" t="n">
         <v>46042</v>
       </c>
-      <c r="S1" s="2" t="n">
+      <c r="S1" s="1" t="n">
         <v>46043</v>
       </c>
-      <c r="T1" s="2" t="n">
+      <c r="T1" s="1" t="n">
         <v>46044</v>
       </c>
-      <c r="U1" s="2" t="n">
+      <c r="U1" s="1" t="n">
         <v>46045</v>
       </c>
-      <c r="V1" s="2" t="n">
+      <c r="V1" s="1" t="n">
         <v>46046</v>
       </c>
-      <c r="W1" s="2" t="n">
+      <c r="W1" s="1" t="n">
         <v>46047</v>
       </c>
-      <c r="X1" s="2" t="n">
+      <c r="X1" s="1" t="n">
         <v>46048</v>
       </c>
-      <c r="Y1" s="2" t="n">
+      <c r="Y1" s="1" t="n">
         <v>46049</v>
       </c>
-      <c r="Z1" s="2" t="n">
+      <c r="Z1" s="1" t="n">
         <v>46050</v>
       </c>
-      <c r="AA1" s="2" t="n">
+      <c r="AA1" s="1" t="n">
         <v>46051</v>
       </c>
-      <c r="AB1" s="2" t="n">
+      <c r="AB1" s="1" t="n">
         <v>46052</v>
       </c>
-      <c r="AC1" s="2" t="n">
+      <c r="AC1" s="1" t="n">
         <v>46053</v>
       </c>
-      <c r="AD1" s="2" t="n">
+      <c r="AD1" s="1" t="n">
         <v>46054</v>
       </c>
-      <c r="AE1" s="2" t="n">
+      <c r="AE1" s="1" t="n">
         <v>46055</v>
       </c>
-      <c r="AF1" s="2" t="n">
+      <c r="AF1" s="1" t="n">
         <v>46056</v>
       </c>
-      <c r="AG1" s="2" t="n">
+      <c r="AG1" s="1" t="n">
         <v>46057</v>
       </c>
-      <c r="AH1" s="2" t="n">
+      <c r="AH1" s="1" t="n">
         <v>46058</v>
       </c>
-      <c r="AI1" s="2" t="n">
+      <c r="AI1" s="1" t="n">
         <v>46059</v>
       </c>
-      <c r="AJ1" s="2" t="n">
+      <c r="AJ1" s="1" t="n">
         <v>46060</v>
       </c>
-      <c r="AK1" s="2" t="n">
+      <c r="AK1" s="1" t="n">
         <v>46061</v>
       </c>
-      <c r="AL1" s="2" t="n">
+      <c r="AL1" s="1" t="n">
         <v>46062</v>
       </c>
-      <c r="AM1" s="2" t="n">
+      <c r="AM1" s="1" t="n">
         <v>46063</v>
       </c>
-      <c r="AN1" s="2" t="n">
+      <c r="AN1" s="1" t="n">
         <v>46064</v>
       </c>
-      <c r="AO1" s="2" t="n">
+      <c r="AO1" s="1" t="n">
         <v>46065</v>
       </c>
-      <c r="AP1" s="2" t="n">
+      <c r="AP1" s="1" t="n">
         <v>46066</v>
       </c>
-      <c r="AQ1" s="2" t="n">
+      <c r="AQ1" s="1" t="n">
         <v>46067</v>
       </c>
-      <c r="AR1" s="2" t="n">
+      <c r="AR1" s="1" t="n">
         <v>46068</v>
       </c>
-      <c r="AS1" s="2" t="n">
+      <c r="AS1" s="1" t="n">
         <v>46069</v>
       </c>
-      <c r="AT1" s="2" t="n">
+      <c r="AT1" s="1" t="n">
         <v>46070</v>
       </c>
-      <c r="AU1" s="2" t="n">
+      <c r="AU1" s="1" t="n">
         <v>46071</v>
       </c>
-      <c r="AV1" s="2" t="n">
+      <c r="AV1" s="1" t="n">
         <v>46072</v>
       </c>
-      <c r="AW1" s="2" t="n">
+      <c r="AW1" s="1" t="n">
         <v>46073</v>
       </c>
-      <c r="AX1" s="2" t="n">
+      <c r="AX1" s="1" t="n">
         <v>46074</v>
       </c>
-      <c r="AY1" s="2" t="n">
+      <c r="AY1" s="1" t="n">
         <v>46075</v>
       </c>
-      <c r="AZ1" s="2" t="n">
+      <c r="AZ1" s="1" t="n">
         <v>46076</v>
       </c>
-      <c r="BA1" s="2" t="n">
+      <c r="BA1" s="1" t="n">
         <v>46077</v>
       </c>
-      <c r="BB1" s="2" t="n">
+      <c r="BB1" s="1" t="n">
         <v>46078</v>
       </c>
-      <c r="BC1" s="2" t="n">
+      <c r="BC1" s="1" t="n">
         <v>46079</v>
       </c>
-      <c r="BD1" s="2" t="n">
+      <c r="BD1" s="1" t="n">
         <v>46080</v>
       </c>
-      <c r="BE1" s="2" t="n">
+      <c r="BE1" s="1" t="n">
         <v>46081</v>
       </c>
-      <c r="BF1" s="2" t="n">
+      <c r="BF1" s="1" t="n">
         <v>46082</v>
       </c>
-      <c r="BG1" s="2" t="n">
+      <c r="BG1" s="1" t="n">
         <v>46083</v>
       </c>
-      <c r="BH1" s="2" t="n">
+      <c r="BH1" s="1" t="n">
         <v>46084</v>
       </c>
-      <c r="BI1" s="2" t="n">
+      <c r="BI1" s="1" t="n">
         <v>46085</v>
       </c>
-      <c r="BJ1" s="2" t="n">
+      <c r="BJ1" s="1" t="n">
         <v>46086</v>
       </c>
-      <c r="BK1" s="2" t="n">
+      <c r="BK1" s="1" t="n">
         <v>46087</v>
       </c>
-      <c r="BL1" s="2" t="n">
+      <c r="BL1" s="1" t="n">
         <v>46088</v>
       </c>
-      <c r="BM1" s="2" t="n">
+      <c r="BM1" s="1" t="n">
         <v>46089</v>
       </c>
-      <c r="BN1" s="2" t="n">
+      <c r="BN1" s="1" t="n">
         <v>46090</v>
       </c>
-      <c r="BO1" s="2" t="n">
+      <c r="BO1" s="1" t="n">
         <v>46091</v>
       </c>
-      <c r="BP1" s="2" t="n">
+      <c r="BP1" s="1" t="n">
         <v>46092</v>
       </c>
-      <c r="BQ1" s="2" t="n">
+      <c r="BQ1" s="1" t="n">
         <v>46093</v>
       </c>
-      <c r="BR1" s="2" t="n">
+      <c r="BR1" s="1" t="n">
         <v>46094</v>
       </c>
-      <c r="BS1" s="2" t="n">
+      <c r="BS1" s="1" t="n">
         <v>46095</v>
       </c>
-      <c r="BT1" s="2" t="n">
+      <c r="BT1" s="1" t="n">
         <v>46096</v>
       </c>
-      <c r="BU1" s="2" t="n">
+      <c r="BU1" s="1" t="n">
         <v>46097</v>
       </c>
-      <c r="BV1" s="2" t="n">
+      <c r="BV1" s="1" t="n">
         <v>46098</v>
       </c>
-      <c r="BW1" s="2" t="n">
+      <c r="BW1" s="1" t="n">
         <v>46099</v>
       </c>
-      <c r="BX1" s="2" t="n">
+      <c r="BX1" s="1" t="n">
         <v>46100</v>
       </c>
-      <c r="BY1" s="2" t="n">
+      <c r="BY1" s="1" t="n">
         <v>46101</v>
       </c>
-      <c r="BZ1" s="2" t="n">
+      <c r="BZ1" s="1" t="n">
         <v>46102</v>
       </c>
-      <c r="CA1" s="2" t="n">
+      <c r="CA1" s="1" t="n">
         <v>46103</v>
       </c>
-      <c r="CB1" s="2" t="n">
+      <c r="CB1" s="1" t="n">
         <v>46104</v>
       </c>
-      <c r="CC1" s="2" t="n">
+      <c r="CC1" s="1" t="n">
         <v>46105</v>
       </c>
-      <c r="CD1" s="2" t="n">
+      <c r="CD1" s="1" t="n">
         <v>46106</v>
       </c>
-      <c r="CE1" s="2" t="n">
+      <c r="CE1" s="1" t="n">
         <v>46107</v>
       </c>
-      <c r="CF1" s="2" t="n">
+      <c r="CF1" s="1" t="n">
         <v>46108</v>
       </c>
-      <c r="CG1" s="2" t="n">
+      <c r="CG1" s="1" t="n">
         <v>46109</v>
       </c>
-      <c r="CH1" s="2" t="n">
+      <c r="CH1" s="1" t="n">
         <v>46110</v>
       </c>
-      <c r="CI1" s="2" t="n">
+      <c r="CI1" s="1" t="n">
         <v>46111</v>
       </c>
-      <c r="CJ1" s="2" t="n">
+      <c r="CJ1" s="1" t="n">
         <v>46112</v>
       </c>
-      <c r="CK1" s="2" t="n">
-        <v>46023</v>
-      </c>
-      <c r="CL1" s="2" t="n">
-        <v>46024</v>
-      </c>
-      <c r="CM1" s="2" t="n">
-        <v>46025</v>
-      </c>
-      <c r="CN1" s="2" t="n">
-        <v>46026</v>
-      </c>
-      <c r="CO1" s="2" t="n">
-        <v>46027</v>
-      </c>
-      <c r="CP1" s="2" t="n">
-        <v>46028</v>
-      </c>
-      <c r="CQ1" s="2" t="n">
+      <c r="CK1" s="1" t="n">
         <v>46113</v>
       </c>
-      <c r="CR1" s="2" t="n">
+      <c r="CL1" s="1" t="n">
         <v>46114</v>
       </c>
-      <c r="CS1" s="2" t="n">
+      <c r="CM1" s="1" t="n">
         <v>46115</v>
       </c>
-      <c r="CT1" s="2" t="n">
+      <c r="CN1" s="1" t="n">
         <v>46116</v>
       </c>
-      <c r="CU1" s="2" t="n">
+      <c r="CO1" s="1" t="n">
         <v>46117</v>
       </c>
-      <c r="CV1" s="2" t="n">
+      <c r="CP1" s="1" t="n">
         <v>46118</v>
       </c>
-      <c r="CW1" s="2" t="n">
+      <c r="CQ1" s="1" t="n">
         <v>46119</v>
       </c>
-      <c r="CX1" s="2" t="n">
+      <c r="CR1" s="1" t="n">
         <v>46120</v>
       </c>
-      <c r="CY1" s="2" t="n">
+      <c r="CS1" s="1" t="n">
         <v>46121</v>
       </c>
-      <c r="CZ1" s="2" t="n">
+      <c r="CT1" s="1" t="n">
         <v>46122</v>
       </c>
-      <c r="DA1" s="2" t="n">
+      <c r="CU1" s="1" t="n">
         <v>46123</v>
       </c>
-      <c r="DB1" s="2" t="n">
+      <c r="CV1" s="1" t="n">
         <v>46124</v>
       </c>
-      <c r="DC1" s="2" t="n">
+      <c r="CW1" s="1" t="n">
         <v>46125</v>
       </c>
-      <c r="DD1" s="2" t="n">
+      <c r="CX1" s="1" t="n">
         <v>46126</v>
       </c>
-      <c r="DE1" s="2" t="n">
+      <c r="CY1" s="1" t="n">
         <v>46127</v>
       </c>
-      <c r="DF1" s="2" t="n">
+      <c r="CZ1" s="1" t="n">
         <v>46128</v>
       </c>
-      <c r="DG1" s="2" t="n">
+      <c r="DA1" s="1" t="n">
         <v>46129</v>
       </c>
-      <c r="DH1" s="2" t="n">
+      <c r="DB1" s="1" t="n">
         <v>46130</v>
       </c>
-      <c r="DI1" s="2" t="n">
+      <c r="DC1" s="1" t="n">
         <v>46131</v>
       </c>
-      <c r="DJ1" s="2" t="n">
+      <c r="DD1" s="1" t="n">
         <v>46132</v>
       </c>
-      <c r="DK1" s="2" t="n">
+      <c r="DE1" s="1" t="n">
         <v>46133</v>
       </c>
-      <c r="DL1" s="2" t="n">
+      <c r="DF1" s="1" t="n">
         <v>46134</v>
       </c>
-      <c r="DM1" s="2" t="n">
+      <c r="DG1" s="1" t="n">
         <v>46135</v>
       </c>
-      <c r="DN1" s="2" t="n">
+      <c r="DH1" s="1" t="n">
         <v>46136</v>
       </c>
-      <c r="DO1" s="2" t="n">
+      <c r="DI1" s="1" t="n">
         <v>46137</v>
       </c>
-      <c r="DP1" s="2" t="n">
+      <c r="DJ1" s="1" t="n">
         <v>46138</v>
       </c>
-      <c r="DQ1" s="2" t="n">
+      <c r="DK1" s="1" t="n">
         <v>46139</v>
       </c>
-      <c r="DR1" s="2" t="n">
+      <c r="DL1" s="1" t="n">
         <v>46140</v>
       </c>
-      <c r="DS1" s="2" t="n">
+      <c r="DM1" s="1" t="n">
         <v>46141</v>
       </c>
-      <c r="DT1" s="2" t="n">
+      <c r="DN1" s="1" t="n">
         <v>46142</v>
       </c>
-      <c r="DU1" s="2" t="n">
+      <c r="DO1" s="1" t="n">
         <v>46143</v>
       </c>
-      <c r="DV1" s="2" t="n">
+      <c r="DP1" s="1" t="n">
         <v>46144</v>
       </c>
-      <c r="DW1" s="2" t="n">
+      <c r="DQ1" s="1" t="n">
         <v>46145</v>
       </c>
-      <c r="DX1" s="2" t="n">
+      <c r="DR1" s="1" t="n">
         <v>46146</v>
       </c>
-      <c r="DY1" s="2" t="n">
+      <c r="DS1" s="1" t="n">
         <v>46147</v>
       </c>
-      <c r="DZ1" s="2" t="n">
+      <c r="DT1" s="1" t="n">
         <v>46148</v>
       </c>
-      <c r="EA1" s="2" t="n">
+      <c r="DU1" s="1" t="n">
         <v>46149</v>
       </c>
-      <c r="EB1" s="2" t="n">
+      <c r="DV1" s="1" t="n">
         <v>46150</v>
       </c>
-      <c r="EC1" s="2" t="n">
+      <c r="DW1" s="1" t="n">
         <v>46151</v>
       </c>
-      <c r="ED1" s="2" t="n">
+      <c r="DX1" s="1" t="n">
         <v>46152</v>
       </c>
-      <c r="EE1" s="2" t="n">
+      <c r="DY1" s="1" t="n">
         <v>46153</v>
       </c>
-      <c r="EF1" s="2" t="n">
+      <c r="DZ1" s="1" t="n">
         <v>46154</v>
       </c>
-      <c r="EG1" s="2" t="n">
+      <c r="EA1" s="1" t="n">
         <v>46155</v>
       </c>
-      <c r="EH1" s="2" t="n">
+      <c r="EB1" s="1" t="n">
         <v>46156</v>
       </c>
-      <c r="EI1" s="2" t="n">
+      <c r="EC1" s="1" t="n">
         <v>46157</v>
       </c>
-      <c r="EJ1" s="2" t="n">
+      <c r="ED1" s="1" t="n">
         <v>46158</v>
       </c>
-      <c r="EK1" s="2" t="n">
+      <c r="EE1" s="1" t="n">
         <v>46159</v>
       </c>
-      <c r="EL1" s="2" t="n">
+      <c r="EF1" s="1" t="n">
         <v>46160</v>
       </c>
-      <c r="EM1" s="2" t="n">
+      <c r="EG1" s="1" t="n">
         <v>46161</v>
       </c>
-      <c r="EN1" s="2" t="n">
+      <c r="EH1" s="1" t="n">
         <v>46162</v>
       </c>
-      <c r="EO1" s="2" t="n">
+      <c r="EI1" s="1" t="n">
         <v>46163</v>
       </c>
-      <c r="EP1" s="2" t="n">
+      <c r="EJ1" s="1" t="n">
         <v>46164</v>
       </c>
-      <c r="EQ1" s="2" t="n">
+      <c r="EK1" s="1" t="n">
         <v>46165</v>
       </c>
-      <c r="ER1" s="2" t="n">
+      <c r="EL1" s="1" t="n">
         <v>46166</v>
       </c>
-      <c r="ES1" s="2" t="n">
+      <c r="EM1" s="1" t="n">
         <v>46167</v>
       </c>
-      <c r="ET1" s="2" t="n">
+      <c r="EN1" s="1" t="n">
         <v>46168</v>
       </c>
-      <c r="EU1" s="2" t="n">
+      <c r="EO1" s="1" t="n">
         <v>46169</v>
       </c>
-      <c r="EV1" s="2" t="n">
+      <c r="EP1" s="1" t="n">
         <v>46170</v>
       </c>
-      <c r="EW1" s="2" t="n">
+      <c r="EQ1" s="1" t="n">
         <v>46171</v>
       </c>
-      <c r="EX1" s="2" t="n">
+      <c r="ER1" s="1" t="n">
         <v>46172</v>
       </c>
-      <c r="EY1" s="2" t="n">
+      <c r="ES1" s="1" t="n">
         <v>46173</v>
-      </c>
-      <c r="EZ1" s="6" t="n">
-        <v>46022</v>
       </c>
     </row>
     <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Supervisor</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr">
+        <is>
+          <t>Jairo Porras</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>T258</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Fuel Attendant</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Juan Steven</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>L159</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Supervisor</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Jairo Porras</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>T258</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Fuel Attendant</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Vincent Rolong</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>K789</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Carga inicial de version QAV2
</commit_message>
<xml_diff>
--- a/PlanStaffRGM.xlsx
+++ b/PlanStaffRGM.xlsx
@@ -28,12 +28,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00AA5500"/>
+        <bgColor rgb="00AA5500"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -48,9 +60,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -125,6 +139,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>ShiftType</author>
+  </authors>
+  <commentList>
+    <comment ref="AL3" authorId="0" shapeId="0">
+      <text>
+        <t>07:00-16:00</t>
+      </text>
+    </comment>
+    <comment ref="AM3" authorId="0" shapeId="0">
+      <text>
+        <t>07:00-16:00</t>
+      </text>
+    </comment>
+    <comment ref="AN3" authorId="0" shapeId="0">
+      <text>
+        <t>07:00-16:00</t>
+      </text>
+    </comment>
+    <comment ref="AO3" authorId="0" shapeId="0">
+      <text>
+        <t>07:00-16:00</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -877,38 +921,79 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Supervisor</t>
+          <t>Fuel Attendant</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Jairo Porras</t>
+          <t>Juan David</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>T258</t>
+          <t>M236</t>
+        </is>
+      </c>
+      <c r="AL2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AM2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AN2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AO2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Fuel Attendant</t>
+          <t>Supervisor</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Juan Steven</t>
+          <t>Alejandro</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>L159</t>
+          <t>N596</t>
+        </is>
+      </c>
+      <c r="AL3" s="3" t="inlineStr">
+        <is>
+          <t>E16</t>
+        </is>
+      </c>
+      <c r="AM3" s="3" t="inlineStr">
+        <is>
+          <t>E16</t>
+        </is>
+      </c>
+      <c r="AN3" s="3" t="inlineStr">
+        <is>
+          <t>E16</t>
+        </is>
+      </c>
+      <c r="AO3" s="3" t="inlineStr">
+        <is>
+          <t>E16</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
falta mejorar un caso de uso al copiar y pegar ON y ON NS
</commit_message>
<xml_diff>
--- a/PlanStaffRGM.xlsx
+++ b/PlanStaffRGM.xlsx
@@ -27,7 +27,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -58,6 +58,18 @@
         <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00AA0000"/>
+        <bgColor rgb="00AA0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0055FFFF"/>
+        <bgColor rgb="0055FFFF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -71,13 +83,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -160,11 +174,6 @@
     <author>ShiftType</author>
   </authors>
   <commentList>
-    <comment ref="H2" authorId="0" shapeId="0">
-      <text>
-        <t>07:00-13:00</t>
-      </text>
-    </comment>
     <comment ref="I2" authorId="0" shapeId="0">
       <text>
         <t>07:00-13:00</t>
@@ -175,34 +184,34 @@
         <t>07:00-13:00</t>
       </text>
     </comment>
-    <comment ref="P2" authorId="0" shapeId="0">
+    <comment ref="K2" authorId="0" shapeId="0">
       <text>
         <t>07:00-13:00</t>
       </text>
     </comment>
-    <comment ref="Q2" authorId="0" shapeId="0">
+    <comment ref="L2" authorId="0" shapeId="0">
       <text>
         <t>07:00-13:00</t>
       </text>
     </comment>
-    <comment ref="S2" authorId="0" shapeId="0">
+    <comment ref="O2" authorId="0" shapeId="0">
       <text>
-        <t>07:00-13:00</t>
+        <t>04:00-17:00</t>
       </text>
     </comment>
-    <comment ref="T2" authorId="0" shapeId="0">
+    <comment ref="P2" authorId="0" shapeId="0">
       <text>
-        <t>07:00-13:00</t>
+        <t>04:00-17:00</t>
       </text>
     </comment>
-    <comment ref="U2" authorId="0" shapeId="0">
+    <comment ref="EW2" authorId="0" shapeId="0">
       <text>
-        <t>07:00-13:00</t>
+        <t>04:00-17:00</t>
       </text>
     </comment>
-    <comment ref="EV2" authorId="0" shapeId="0">
+    <comment ref="EX2" authorId="0" shapeId="0">
       <text>
-        <t>07:00-13:00</t>
+        <t>04:00-17:00</t>
       </text>
     </comment>
   </commentList>
@@ -1007,174 +1016,94 @@
           <t>ON</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>ONH</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>ONH</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>ONH</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>ONH</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="N2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="O2" s="6" t="inlineStr">
+        <is>
+          <t>WH</t>
+        </is>
+      </c>
+      <c r="P2" s="6" t="inlineStr">
+        <is>
+          <t>WH</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="R2" s="3" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="S2" s="3" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="T2" s="3" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="ET2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="EU2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="EV2" s="2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="O2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="P2" s="4" t="inlineStr">
-        <is>
-          <t>ONH</t>
-        </is>
-      </c>
-      <c r="Q2" s="4" t="inlineStr">
-        <is>
-          <t>ONH</t>
-        </is>
-      </c>
-      <c r="R2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="S2" s="4" t="inlineStr">
-        <is>
-          <t>ONH</t>
-        </is>
-      </c>
-      <c r="T2" s="4" t="inlineStr">
-        <is>
-          <t>ONH</t>
-        </is>
-      </c>
-      <c r="U2" s="4" t="inlineStr">
-        <is>
-          <t>ONH</t>
-        </is>
-      </c>
-      <c r="V2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="W2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="X2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="Y2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="Z2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AA2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AB2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AZ2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="BA2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="BB2" s="3" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="BC2" s="3" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="BD2" s="3" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="BE2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BF2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BG2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="ET2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="EU2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="EV2" s="4" t="inlineStr">
-        <is>
-          <t>ONH</t>
-        </is>
-      </c>
-      <c r="EW2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="EX2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
+      <c r="EW2" s="6" t="inlineStr">
+        <is>
+          <t>WH</t>
+        </is>
+      </c>
+      <c r="EX2" s="6" t="inlineStr">
+        <is>
+          <t>WH</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
actualmente esta tomando son las horas del ON u ON NS que se copio, hacer correcion de esto o dejarlo asi pero sin preguntar la hora a insertar
</commit_message>
<xml_diff>
--- a/PlanStaffRGM.xlsx
+++ b/PlanStaffRGM.xlsx
@@ -174,44 +174,49 @@
     <author>ShiftType</author>
   </authors>
   <commentList>
+    <comment ref="H2" authorId="0" shapeId="0">
+      <text>
+        <t>04:00-17:00</t>
+      </text>
+    </comment>
     <comment ref="I2" authorId="0" shapeId="0">
+      <text>
+        <t>04:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="J2" authorId="0" shapeId="0">
+      <text>
+        <t>04:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="K2" authorId="0" shapeId="0">
+      <text>
+        <t>04:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="O2" authorId="0" shapeId="0">
       <text>
         <t>07:00-13:00</t>
       </text>
     </comment>
-    <comment ref="J2" authorId="0" shapeId="0">
+    <comment ref="ET2" authorId="0" shapeId="0">
       <text>
         <t>07:00-13:00</t>
       </text>
     </comment>
-    <comment ref="K2" authorId="0" shapeId="0">
+    <comment ref="EU2" authorId="0" shapeId="0">
       <text>
         <t>07:00-13:00</t>
       </text>
     </comment>
-    <comment ref="L2" authorId="0" shapeId="0">
+    <comment ref="EV2" authorId="0" shapeId="0">
       <text>
         <t>07:00-13:00</t>
       </text>
     </comment>
-    <comment ref="O2" authorId="0" shapeId="0">
-      <text>
-        <t>04:00-17:00</t>
-      </text>
-    </comment>
-    <comment ref="P2" authorId="0" shapeId="0">
-      <text>
-        <t>04:00-17:00</t>
-      </text>
-    </comment>
     <comment ref="EW2" authorId="0" shapeId="0">
       <text>
-        <t>04:00-17:00</t>
-      </text>
-    </comment>
-    <comment ref="EX2" authorId="0" shapeId="0">
-      <text>
-        <t>04:00-17:00</t>
+        <t>07:00-13:00</t>
       </text>
     </comment>
   </commentList>
@@ -1016,94 +1021,74 @@
           <t>ON</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>WH</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>WH</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="inlineStr">
+        <is>
+          <t>WH</t>
+        </is>
+      </c>
+      <c r="K2" s="6" t="inlineStr">
+        <is>
+          <t>WH</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="N2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="O2" s="4" t="inlineStr">
+        <is>
+          <t>ONH</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ET2" s="4" t="inlineStr">
         <is>
           <t>ONH</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="EU2" s="4" t="inlineStr">
         <is>
           <t>ONH</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="EV2" s="4" t="inlineStr">
         <is>
           <t>ONH</t>
         </is>
       </c>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="EW2" s="4" t="inlineStr">
         <is>
           <t>ONH</t>
-        </is>
-      </c>
-      <c r="M2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="N2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="O2" s="6" t="inlineStr">
-        <is>
-          <t>WH</t>
-        </is>
-      </c>
-      <c r="P2" s="6" t="inlineStr">
-        <is>
-          <t>WH</t>
-        </is>
-      </c>
-      <c r="Q2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="R2" s="3" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="S2" s="3" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="T2" s="3" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="ET2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="EU2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="EV2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="EW2" s="6" t="inlineStr">
-        <is>
-          <t>WH</t>
-        </is>
-      </c>
-      <c r="EX2" s="6" t="inlineStr">
-        <is>
-          <t>WH</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
software 100 % funcional, despues de este commit se testeara con plan staff real de inbound outbound
</commit_message>
<xml_diff>
--- a/PlanStaffRGM.xlsx
+++ b/PlanStaffRGM.xlsx
@@ -189,12 +189,22 @@
         <t>04:00-17:00</t>
       </text>
     </comment>
-    <comment ref="K2" authorId="0" shapeId="0">
+    <comment ref="M2" authorId="0" shapeId="0">
       <text>
-        <t>04:00-17:00</t>
+        <t>07:00-13:00</t>
       </text>
     </comment>
-    <comment ref="O2" authorId="0" shapeId="0">
+    <comment ref="N2" authorId="0" shapeId="0">
+      <text>
+        <t>07:00-13:00</t>
+      </text>
+    </comment>
+    <comment ref="P2" authorId="0" shapeId="0">
+      <text>
+        <t>07:00-13:00</t>
+      </text>
+    </comment>
+    <comment ref="Q2" authorId="0" shapeId="0">
       <text>
         <t>07:00-13:00</t>
       </text>
@@ -204,17 +214,7 @@
         <t>07:00-13:00</t>
       </text>
     </comment>
-    <comment ref="EU2" authorId="0" shapeId="0">
-      <text>
-        <t>07:00-13:00</t>
-      </text>
-    </comment>
     <comment ref="EV2" authorId="0" shapeId="0">
-      <text>
-        <t>07:00-13:00</t>
-      </text>
-    </comment>
-    <comment ref="EW2" authorId="0" shapeId="0">
       <text>
         <t>07:00-13:00</t>
       </text>
@@ -1036,9 +1036,9 @@
           <t>WH</t>
         </is>
       </c>
-      <c r="K2" s="6" t="inlineStr">
-        <is>
-          <t>WH</t>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
       <c r="L2" s="5" t="inlineStr">
@@ -1046,47 +1046,42 @@
           <t>OFF</t>
         </is>
       </c>
-      <c r="M2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="N2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="O2" s="4" t="inlineStr">
+      <c r="M2" s="4" t="inlineStr">
         <is>
           <t>ONH</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="N2" s="4" t="inlineStr">
+        <is>
+          <t>ONH</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="Q2" s="2" t="inlineStr">
+      <c r="P2" s="4" t="inlineStr">
+        <is>
+          <t>ONH</t>
+        </is>
+      </c>
+      <c r="Q2" s="4" t="inlineStr">
+        <is>
+          <t>ONH</t>
+        </is>
+      </c>
+      <c r="ET2" s="4" t="inlineStr">
+        <is>
+          <t>ONH</t>
+        </is>
+      </c>
+      <c r="EU2" s="2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="ET2" s="4" t="inlineStr">
-        <is>
-          <t>ONH</t>
-        </is>
-      </c>
-      <c r="EU2" s="4" t="inlineStr">
-        <is>
-          <t>ONH</t>
-        </is>
-      </c>
       <c r="EV2" s="4" t="inlineStr">
-        <is>
-          <t>ONH</t>
-        </is>
-      </c>
-      <c r="EW2" s="4" t="inlineStr">
         <is>
           <t>ONH</t>
         </is>

</xml_diff>

<commit_message>
unir mismo viaje funcional y separar viajes semifuncional
</commit_message>
<xml_diff>
--- a/PlanStaffRGM.xlsx
+++ b/PlanStaffRGM.xlsx
@@ -174,37 +174,32 @@
     <author>ShiftType</author>
   </authors>
   <commentList>
-    <comment ref="H2" authorId="0" shapeId="0">
-      <text>
-        <t>04:00-17:00</t>
-      </text>
-    </comment>
-    <comment ref="I2" authorId="0" shapeId="0">
-      <text>
-        <t>04:00-17:00</t>
-      </text>
-    </comment>
-    <comment ref="J2" authorId="0" shapeId="0">
-      <text>
-        <t>04:00-17:00</t>
-      </text>
-    </comment>
-    <comment ref="M2" authorId="0" shapeId="0">
+    <comment ref="O2" authorId="0" shapeId="0">
       <text>
         <t>07:00-13:00</t>
       </text>
     </comment>
-    <comment ref="N2" authorId="0" shapeId="0">
+    <comment ref="R2" authorId="0" shapeId="0">
       <text>
         <t>07:00-13:00</t>
       </text>
     </comment>
-    <comment ref="P2" authorId="0" shapeId="0">
+    <comment ref="U2" authorId="0" shapeId="0">
       <text>
         <t>07:00-13:00</t>
       </text>
     </comment>
-    <comment ref="Q2" authorId="0" shapeId="0">
+    <comment ref="V2" authorId="0" shapeId="0">
+      <text>
+        <t>07:00-13:00</t>
+      </text>
+    </comment>
+    <comment ref="W2" authorId="0" shapeId="0">
+      <text>
+        <t>07:00-13:00</t>
+      </text>
+    </comment>
+    <comment ref="X2" authorId="0" shapeId="0">
       <text>
         <t>07:00-13:00</t>
       </text>
@@ -214,7 +209,22 @@
         <t>07:00-13:00</t>
       </text>
     </comment>
+    <comment ref="EU2" authorId="0" shapeId="0">
+      <text>
+        <t>07:00-13:00</t>
+      </text>
+    </comment>
     <comment ref="EV2" authorId="0" shapeId="0">
+      <text>
+        <t>07:00-13:00</t>
+      </text>
+    </comment>
+    <comment ref="EW2" authorId="0" shapeId="0">
+      <text>
+        <t>07:00-13:00</t>
+      </text>
+    </comment>
+    <comment ref="EX2" authorId="0" shapeId="0">
       <text>
         <t>07:00-13:00</t>
       </text>
@@ -1021,19 +1031,19 @@
           <t>ON</t>
         </is>
       </c>
-      <c r="H2" s="6" t="inlineStr">
-        <is>
-          <t>WH</t>
-        </is>
-      </c>
-      <c r="I2" s="6" t="inlineStr">
-        <is>
-          <t>WH</t>
-        </is>
-      </c>
-      <c r="J2" s="6" t="inlineStr">
-        <is>
-          <t>WH</t>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
@@ -1046,42 +1056,87 @@
           <t>OFF</t>
         </is>
       </c>
-      <c r="M2" s="4" t="inlineStr">
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="N2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="O2" s="4" t="inlineStr">
         <is>
           <t>ONH</t>
         </is>
       </c>
-      <c r="N2" s="4" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R2" s="4" t="inlineStr">
         <is>
           <t>ONH</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="S2" s="2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="P2" s="4" t="inlineStr">
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="U2" s="4" t="inlineStr">
         <is>
           <t>ONH</t>
         </is>
       </c>
-      <c r="Q2" s="4" t="inlineStr">
+      <c r="V2" s="4" t="inlineStr">
         <is>
           <t>ONH</t>
         </is>
       </c>
+      <c r="W2" s="4" t="inlineStr">
+        <is>
+          <t>ONH</t>
+        </is>
+      </c>
+      <c r="X2" s="4" t="inlineStr">
+        <is>
+          <t>ONH</t>
+        </is>
+      </c>
       <c r="ET2" s="4" t="inlineStr">
         <is>
           <t>ONH</t>
         </is>
       </c>
-      <c r="EU2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
+      <c r="EU2" s="4" t="inlineStr">
+        <is>
+          <t>ONH</t>
         </is>
       </c>
       <c r="EV2" s="4" t="inlineStr">
+        <is>
+          <t>ONH</t>
+        </is>
+      </c>
+      <c r="EW2" s="4" t="inlineStr">
+        <is>
+          <t>ONH</t>
+        </is>
+      </c>
+      <c r="EX2" s="4" t="inlineStr">
         <is>
           <t>ONH</t>
         </is>

</xml_diff>

<commit_message>
codigo con solucion asociada al drag al 100%, sera sometido a testing completo
</commit_message>
<xml_diff>
--- a/PlanStaffRGM.xlsx
+++ b/PlanStaffRGM.xlsx
@@ -174,13 +174,48 @@
     <author>ShiftType</author>
   </authors>
   <commentList>
-    <comment ref="O2" authorId="0" shapeId="0">
+    <comment ref="H2" authorId="0" shapeId="0">
+      <text>
+        <t>04:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="I2" authorId="0" shapeId="0">
+      <text>
+        <t>04:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="J2" authorId="0" shapeId="0">
+      <text>
+        <t>04:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="K2" authorId="0" shapeId="0">
+      <text>
+        <t>04:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="P2" authorId="0" shapeId="0">
       <text>
         <t>07:00-13:00</t>
       </text>
     </comment>
+    <comment ref="Q2" authorId="0" shapeId="0">
+      <text>
+        <t>07:00-13:00</t>
+      </text>
+    </comment>
     <comment ref="R2" authorId="0" shapeId="0">
       <text>
+        <t>00:00-00:00</t>
+      </text>
+    </comment>
+    <comment ref="S2" authorId="0" shapeId="0">
+      <text>
+        <t>00:00-00:00</t>
+      </text>
+    </comment>
+    <comment ref="T2" authorId="0" shapeId="0">
+      <text>
         <t>07:00-13:00</t>
       </text>
     </comment>
@@ -189,44 +224,34 @@
         <t>07:00-13:00</t>
       </text>
     </comment>
-    <comment ref="V2" authorId="0" shapeId="0">
+    <comment ref="X2" authorId="0" shapeId="0">
       <text>
         <t>07:00-13:00</t>
       </text>
     </comment>
-    <comment ref="W2" authorId="0" shapeId="0">
+    <comment ref="Y2" authorId="0" shapeId="0">
       <text>
         <t>07:00-13:00</t>
       </text>
     </comment>
-    <comment ref="X2" authorId="0" shapeId="0">
+    <comment ref="Z2" authorId="0" shapeId="0">
       <text>
         <t>07:00-13:00</t>
       </text>
     </comment>
-    <comment ref="ET2" authorId="0" shapeId="0">
+    <comment ref="EV2" authorId="0" shapeId="0">
       <text>
         <t>07:00-13:00</t>
       </text>
     </comment>
-    <comment ref="EU2" authorId="0" shapeId="0">
-      <text>
-        <t>07:00-13:00</t>
-      </text>
-    </comment>
-    <comment ref="EV2" authorId="0" shapeId="0">
-      <text>
-        <t>07:00-13:00</t>
-      </text>
-    </comment>
     <comment ref="EW2" authorId="0" shapeId="0">
       <text>
-        <t>07:00-13:00</t>
+        <t>00:00-00:00</t>
       </text>
     </comment>
     <comment ref="EX2" authorId="0" shapeId="0">
       <text>
-        <t>07:00-13:00</t>
+        <t>00:00-00:00</t>
       </text>
     </comment>
   </commentList>
@@ -522,7 +547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EX2"/>
+  <dimension ref="A1:EX3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -1031,114 +1056,141 @@
           <t>ON</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>WH</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>WH</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="inlineStr">
+        <is>
+          <t>WH</t>
+        </is>
+      </c>
+      <c r="K2" s="6" t="inlineStr">
+        <is>
+          <t>WH</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="N2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="P2" s="4" t="inlineStr">
+        <is>
+          <t>ONH</t>
+        </is>
+      </c>
+      <c r="Q2" s="4" t="inlineStr">
+        <is>
+          <t>ONH</t>
+        </is>
+      </c>
+      <c r="R2" s="7" t="inlineStr">
+        <is>
+          <t>RT</t>
+        </is>
+      </c>
+      <c r="S2" s="7" t="inlineStr">
+        <is>
+          <t>RT</t>
+        </is>
+      </c>
+      <c r="T2" s="4" t="inlineStr">
+        <is>
+          <t>ONH</t>
+        </is>
+      </c>
+      <c r="U2" s="4" t="inlineStr">
+        <is>
+          <t>ONH</t>
+        </is>
+      </c>
+      <c r="V2" s="2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="W2" s="2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="J2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="K2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="L2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="M2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="N2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="O2" s="4" t="inlineStr">
+      <c r="X2" s="4" t="inlineStr">
         <is>
           <t>ONH</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="Q2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="R2" s="4" t="inlineStr">
+      <c r="Y2" s="4" t="inlineStr">
         <is>
           <t>ONH</t>
         </is>
       </c>
-      <c r="S2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="T2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="U2" s="4" t="inlineStr">
+      <c r="Z2" s="4" t="inlineStr">
         <is>
           <t>ONH</t>
         </is>
       </c>
-      <c r="V2" s="4" t="inlineStr">
+      <c r="ET2" s="3" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="EU2" s="3" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="EV2" s="4" t="inlineStr">
         <is>
           <t>ONH</t>
         </is>
       </c>
-      <c r="W2" s="4" t="inlineStr">
-        <is>
-          <t>ONH</t>
-        </is>
-      </c>
-      <c r="X2" s="4" t="inlineStr">
-        <is>
-          <t>ONH</t>
-        </is>
-      </c>
-      <c r="ET2" s="4" t="inlineStr">
-        <is>
-          <t>ONH</t>
-        </is>
-      </c>
-      <c r="EU2" s="4" t="inlineStr">
-        <is>
-          <t>ONH</t>
-        </is>
-      </c>
-      <c r="EV2" s="4" t="inlineStr">
-        <is>
-          <t>ONH</t>
-        </is>
-      </c>
-      <c r="EW2" s="4" t="inlineStr">
-        <is>
-          <t>ONH</t>
-        </is>
-      </c>
-      <c r="EX2" s="4" t="inlineStr">
-        <is>
-          <t>ONH</t>
+      <c r="EW2" s="7" t="inlineStr">
+        <is>
+          <t>RT</t>
+        </is>
+      </c>
+      <c r="EX2" s="7" t="inlineStr">
+        <is>
+          <t>RT</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Supervisor</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Jose Gomez</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>K78</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
funcional al 100 % y disponible para hacer deploy
</commit_message>
<xml_diff>
--- a/PlanStaffRGM.xlsx
+++ b/PlanStaffRGM.xlsx
@@ -27,7 +27,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -70,6 +70,12 @@
         <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0055007F"/>
+        <bgColor rgb="0055007F"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -83,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -92,6 +98,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -174,24 +181,14 @@
     <author>ShiftType</author>
   </authors>
   <commentList>
-    <comment ref="D2" authorId="0" shapeId="0">
+    <comment ref="M2" authorId="0" shapeId="0">
       <text>
-        <t>00:00-00:00</t>
+        <t>07:00-16:00</t>
       </text>
     </comment>
-    <comment ref="E2" authorId="0" shapeId="0">
+    <comment ref="N2" authorId="0" shapeId="0">
       <text>
-        <t>00:00-00:00</t>
-      </text>
-    </comment>
-    <comment ref="F2" authorId="0" shapeId="0">
-      <text>
-        <t>00:00-00:00</t>
-      </text>
-    </comment>
-    <comment ref="G2" authorId="0" shapeId="0">
-      <text>
-        <t>00:00-00:00</t>
+        <t>07:00-16:00</t>
       </text>
     </comment>
     <comment ref="AF2" authorId="0" shapeId="0">
@@ -207,6 +204,66 @@
     <comment ref="AO2" authorId="0" shapeId="0">
       <text>
         <t>07:00-16:00</t>
+      </text>
+    </comment>
+    <comment ref="ET2" authorId="0" shapeId="0">
+      <text>
+        <t>07:00-16:00</t>
+      </text>
+    </comment>
+    <comment ref="D3" authorId="0" shapeId="0">
+      <text>
+        <t>07:00-16:00</t>
+      </text>
+    </comment>
+    <comment ref="E3" authorId="0" shapeId="0">
+      <text>
+        <t>07:00-16:00</t>
+      </text>
+    </comment>
+    <comment ref="H3" authorId="0" shapeId="0">
+      <text>
+        <t>07:00-16:00</t>
+      </text>
+    </comment>
+    <comment ref="I3" authorId="0" shapeId="0">
+      <text>
+        <t>07:00-16:00</t>
+      </text>
+    </comment>
+    <comment ref="J3" authorId="0" shapeId="0">
+      <text>
+        <t>00:00-00:00</t>
+      </text>
+    </comment>
+    <comment ref="K3" authorId="0" shapeId="0">
+      <text>
+        <t>00:00-00:00</t>
+      </text>
+    </comment>
+    <comment ref="L3" authorId="0" shapeId="0">
+      <text>
+        <t>00:00-00:00</t>
+      </text>
+    </comment>
+    <comment ref="D4" authorId="0" shapeId="0">
+      <text>
+        <t>08:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="E4" authorId="0" shapeId="0">
+      <text>
+        <t>08:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="F4" authorId="0" shapeId="0">
+      <text>
+        <t>08:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="G4" authorId="0" shapeId="0">
+      <text>
+        <t>08:00-17:00</t>
       </text>
     </comment>
     <comment ref="AR4" authorId="0" shapeId="0">
@@ -1006,232 +1063,287 @@
           <t>FC-2772</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>E16</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>E16</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AA2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AB2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AC2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AD2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AE2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AF2" s="3" t="inlineStr">
+        <is>
+          <t>E16</t>
+        </is>
+      </c>
+      <c r="AG2" s="4" t="inlineStr">
         <is>
           <t>FUSECON OFFICE</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>FUSECON OFFICE</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>FUSECON OFFICE</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>FUSECON OFFICE</t>
-        </is>
-      </c>
-      <c r="AA2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AB2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AC2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AD2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AE2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AF2" s="3" t="inlineStr">
+      <c r="AH2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AI2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AK2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AL2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AM2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AN2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AO2" s="3" t="inlineStr">
         <is>
           <t>E16</t>
         </is>
       </c>
-      <c r="AG2" s="4" t="inlineStr">
-        <is>
-          <t>FUSECON OFFICE</t>
-        </is>
-      </c>
-      <c r="AH2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AI2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AJ2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AK2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AL2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AM2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AN2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AO2" s="3" t="inlineStr">
+      <c r="AP2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AQ2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AR2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AS2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AT2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AU2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AV2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AW2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AX2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AY2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AZ2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="BA2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="BB2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="BC2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="BD2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="BE2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="BF2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="BG2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="BH2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="BI2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="BJ2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="BK2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="BL2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="BM2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="BN2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="BO2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="BP2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ET2" s="3" t="inlineStr">
         <is>
           <t>E16</t>
         </is>
       </c>
-      <c r="AP2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AQ2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AR2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AS2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AT2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AU2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AV2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AW2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AX2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AY2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AZ2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="BA2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="BB2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="BC2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BD2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BE2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BF2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BG2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BH2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BI2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BJ2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BK2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BL2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BM2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BN2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BO2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BP2" s="2" t="inlineStr">
+      <c r="EU2" s="2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
@@ -1253,6 +1365,51 @@
           <t>FC-2771</t>
         </is>
       </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>E16</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>E16</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>E16</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>E16</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>FUSECON OFFICE</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>FUSECON OFFICE</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>FUSECON OFFICE</t>
+        </is>
+      </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
           <t>ON</t>
@@ -1548,6 +1705,26 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>PRO-9826</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>ND</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>ND</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>ND</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>ND</t>
         </is>
       </c>
       <c r="AJ4" s="2" t="inlineStr">

</xml_diff>

<commit_message>
se hace commit antes del lanzamiento por seguridad
</commit_message>
<xml_diff>
--- a/PlanStaffRGM.xlsx
+++ b/PlanStaffRGM.xlsx
@@ -27,7 +27,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -76,6 +76,18 @@
         <bgColor rgb="0055007F"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00550000"/>
+        <bgColor rgb="00550000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00AA55FF"/>
+        <bgColor rgb="00AA55FF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -89,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -99,6 +111,8 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -181,14 +195,24 @@
     <author>ShiftType</author>
   </authors>
   <commentList>
-    <comment ref="M2" authorId="0" shapeId="0">
+    <comment ref="D2" authorId="0" shapeId="0">
       <text>
-        <t>07:00-16:00</t>
+        <t>06:00-12:00</t>
       </text>
     </comment>
-    <comment ref="N2" authorId="0" shapeId="0">
+    <comment ref="E2" authorId="0" shapeId="0">
       <text>
-        <t>07:00-16:00</t>
+        <t>06:00-12:00</t>
+      </text>
+    </comment>
+    <comment ref="F2" authorId="0" shapeId="0">
+      <text>
+        <t>06:00-12:00</t>
+      </text>
+    </comment>
+    <comment ref="G2" authorId="0" shapeId="0">
+      <text>
+        <t>06:00-12:00</t>
       </text>
     </comment>
     <comment ref="AF2" authorId="0" shapeId="0">
@@ -198,72 +222,12 @@
     </comment>
     <comment ref="AG2" authorId="0" shapeId="0">
       <text>
-        <t>00:00-00:00</t>
+        <t>06:00-12:00</t>
       </text>
     </comment>
     <comment ref="AO2" authorId="0" shapeId="0">
       <text>
         <t>07:00-16:00</t>
-      </text>
-    </comment>
-    <comment ref="ET2" authorId="0" shapeId="0">
-      <text>
-        <t>07:00-16:00</t>
-      </text>
-    </comment>
-    <comment ref="D3" authorId="0" shapeId="0">
-      <text>
-        <t>07:00-16:00</t>
-      </text>
-    </comment>
-    <comment ref="E3" authorId="0" shapeId="0">
-      <text>
-        <t>07:00-16:00</t>
-      </text>
-    </comment>
-    <comment ref="H3" authorId="0" shapeId="0">
-      <text>
-        <t>07:00-16:00</t>
-      </text>
-    </comment>
-    <comment ref="I3" authorId="0" shapeId="0">
-      <text>
-        <t>07:00-16:00</t>
-      </text>
-    </comment>
-    <comment ref="J3" authorId="0" shapeId="0">
-      <text>
-        <t>00:00-00:00</t>
-      </text>
-    </comment>
-    <comment ref="K3" authorId="0" shapeId="0">
-      <text>
-        <t>00:00-00:00</t>
-      </text>
-    </comment>
-    <comment ref="L3" authorId="0" shapeId="0">
-      <text>
-        <t>00:00-00:00</t>
-      </text>
-    </comment>
-    <comment ref="D4" authorId="0" shapeId="0">
-      <text>
-        <t>08:00-17:00</t>
-      </text>
-    </comment>
-    <comment ref="E4" authorId="0" shapeId="0">
-      <text>
-        <t>08:00-17:00</t>
-      </text>
-    </comment>
-    <comment ref="F4" authorId="0" shapeId="0">
-      <text>
-        <t>08:00-17:00</t>
-      </text>
-    </comment>
-    <comment ref="G4" authorId="0" shapeId="0">
-      <text>
-        <t>08:00-17:00</t>
       </text>
     </comment>
     <comment ref="AR4" authorId="0" shapeId="0">
@@ -574,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EX4"/>
+  <dimension ref="A1:EX5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -1063,34 +1027,24 @@
           <t>FC-2772</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="G2" s="6" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="H2" s="6" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="I2" s="6" t="inlineStr">
-        <is>
-          <t>ON NS</t>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>FSC</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>FSC</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>FSC</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>FSC</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
@@ -1108,101 +1062,106 @@
           <t>OFF</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="N2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="O2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="P2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="Q2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AA2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AB2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AC2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AD2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AE2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AF2" s="3" t="inlineStr">
         <is>
           <t>E16</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="AG2" s="9" t="inlineStr">
+        <is>
+          <t>FSC</t>
+        </is>
+      </c>
+      <c r="AH2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AI2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AK2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AL2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AM2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AN2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AO2" s="3" t="inlineStr">
         <is>
           <t>E16</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AA2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AB2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AC2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AD2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AE2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AF2" s="3" t="inlineStr">
-        <is>
-          <t>E16</t>
-        </is>
-      </c>
-      <c r="AG2" s="4" t="inlineStr">
-        <is>
-          <t>FUSECON OFFICE</t>
-        </is>
-      </c>
-      <c r="AH2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AI2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AJ2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AK2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AL2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AM2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AN2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AO2" s="3" t="inlineStr">
-        <is>
-          <t>E16</t>
-        </is>
-      </c>
       <c r="AP2" s="5" t="inlineStr">
         <is>
           <t>OFF</t>
@@ -1338,14 +1297,14 @@
           <t>ON</t>
         </is>
       </c>
-      <c r="ET2" s="3" t="inlineStr">
-        <is>
-          <t>E16</t>
-        </is>
-      </c>
-      <c r="EU2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
+      <c r="ET2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="EU2" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -1365,49 +1324,39 @@
           <t>FC-2771</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>E16</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>E16</t>
-        </is>
-      </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>ON NS</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="I3" s="6" t="inlineStr">
         <is>
           <t>ON NS</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>E16</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>E16</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>FUSECON OFFICE</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>FUSECON OFFICE</t>
-        </is>
-      </c>
-      <c r="L3" s="4" t="inlineStr">
-        <is>
-          <t>FUSECON OFFICE</t>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>ON NS</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
@@ -1707,24 +1656,74 @@
           <t>PRO-9826</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>ND</t>
-        </is>
-      </c>
-      <c r="E4" s="8" t="inlineStr">
-        <is>
-          <t>ND</t>
-        </is>
-      </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>ND</t>
-        </is>
-      </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>ND</t>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
         </is>
       </c>
       <c r="AJ4" s="2" t="inlineStr">
@@ -1890,6 +1889,38 @@
       <c r="BP4" s="6" t="inlineStr">
         <is>
           <t>ON NS</t>
+        </is>
+      </c>
+      <c r="ET4" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="EU4" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="EV4" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Data Analyst</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Vincent Rolong</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>L98</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rama para hacer testing del control z y control y un testing general del software
</commit_message>
<xml_diff>
--- a/PlanStaffRGM.xlsx
+++ b/PlanStaffRGM.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operations_best_opt" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Operations_best_opt" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -187,66 +187,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>ShiftType</author>
-  </authors>
-  <commentList>
-    <comment ref="D2" authorId="0" shapeId="0">
-      <text>
-        <t>06:00-12:00</t>
-      </text>
-    </comment>
-    <comment ref="E2" authorId="0" shapeId="0">
-      <text>
-        <t>06:00-12:00</t>
-      </text>
-    </comment>
-    <comment ref="F2" authorId="0" shapeId="0">
-      <text>
-        <t>06:00-12:00</t>
-      </text>
-    </comment>
-    <comment ref="G2" authorId="0" shapeId="0">
-      <text>
-        <t>06:00-12:00</t>
-      </text>
-    </comment>
-    <comment ref="AF2" authorId="0" shapeId="0">
-      <text>
-        <t>07:00-16:00</t>
-      </text>
-    </comment>
-    <comment ref="AG2" authorId="0" shapeId="0">
-      <text>
-        <t>06:00-12:00</t>
-      </text>
-    </comment>
-    <comment ref="AO2" authorId="0" shapeId="0">
-      <text>
-        <t>07:00-16:00</t>
-      </text>
-    </comment>
-    <comment ref="AR4" authorId="0" shapeId="0">
-      <text>
-        <t>07:00-16:00</t>
-      </text>
-    </comment>
-    <comment ref="AS4" authorId="0" shapeId="0">
-      <text>
-        <t>00:00-00:00</t>
-      </text>
-    </comment>
-    <comment ref="AT4" authorId="0" shapeId="0">
-      <text>
-        <t>00:00-00:00</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1027,256 +967,6 @@
           <t>FC-2772</t>
         </is>
       </c>
-      <c r="D2" s="9" t="inlineStr">
-        <is>
-          <t>FSC</t>
-        </is>
-      </c>
-      <c r="E2" s="9" t="inlineStr">
-        <is>
-          <t>FSC</t>
-        </is>
-      </c>
-      <c r="F2" s="9" t="inlineStr">
-        <is>
-          <t>FSC</t>
-        </is>
-      </c>
-      <c r="G2" s="9" t="inlineStr">
-        <is>
-          <t>FSC</t>
-        </is>
-      </c>
-      <c r="J2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="K2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="L2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="M2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="N2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="O2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="P2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="Q2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AA2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AB2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AC2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AD2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AE2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AF2" s="3" t="inlineStr">
-        <is>
-          <t>E16</t>
-        </is>
-      </c>
-      <c r="AG2" s="9" t="inlineStr">
-        <is>
-          <t>FSC</t>
-        </is>
-      </c>
-      <c r="AH2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AI2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AJ2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AK2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AL2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AM2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AN2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AO2" s="3" t="inlineStr">
-        <is>
-          <t>E16</t>
-        </is>
-      </c>
-      <c r="AP2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AQ2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AR2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AS2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AT2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AU2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AV2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AW2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AX2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AY2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AZ2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="BA2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="BB2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="BC2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BD2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BE2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BF2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BG2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BH2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BI2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BJ2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BK2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BL2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
       <c r="BM2" s="2" t="inlineStr">
         <is>
           <t>ON</t>
@@ -1295,16 +985,6 @@
       <c r="BP2" s="2" t="inlineStr">
         <is>
           <t>ON</t>
-        </is>
-      </c>
-      <c r="ET2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="EU2" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -1324,266 +1004,6 @@
           <t>FC-2771</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="H3" s="6" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="I3" s="6" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="J3" s="6" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="T3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="U3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="V3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="W3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="X3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="Y3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="Z3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AA3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AB3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AC3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AD3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AE3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AF3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AG3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AH3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AI3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AJ3" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AK3" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AL3" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AM3" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AN3" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AO3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AP3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AQ3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AR3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AS3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AT3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AU3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AV3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AW3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AX3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AY3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AZ3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BA3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BB3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BC3" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="BD3" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="BE3" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="BF3" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="BG3" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="BH3" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="BI3" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="BJ3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BK3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BL3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
       <c r="BM3" s="2" t="inlineStr">
         <is>
           <t>ON</t>
@@ -1656,254 +1076,24 @@
           <t>PRO-9826</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="BM4" s="6" t="inlineStr">
         <is>
           <t>ON NS</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="BN4" s="6" t="inlineStr">
         <is>
           <t>ON NS</t>
         </is>
       </c>
-      <c r="J4" s="6" t="inlineStr">
+      <c r="BO4" s="6" t="inlineStr">
         <is>
           <t>ON NS</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="L4" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="M4" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="P4" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="Q4" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AJ4" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AK4" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AL4" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AM4" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AN4" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AO4" s="6" t="inlineStr">
+      <c r="BP4" s="6" t="inlineStr">
         <is>
           <t>ON NS</t>
-        </is>
-      </c>
-      <c r="AP4" s="6" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="AQ4" s="6" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="AR4" s="3" t="inlineStr">
-        <is>
-          <t>E16</t>
-        </is>
-      </c>
-      <c r="AS4" s="7" t="inlineStr">
-        <is>
-          <t>LV</t>
-        </is>
-      </c>
-      <c r="AT4" s="7" t="inlineStr">
-        <is>
-          <t>LV</t>
-        </is>
-      </c>
-      <c r="AU4" s="6" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="AV4" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AW4" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AX4" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AY4" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AZ4" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="BA4" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="BB4" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="BC4" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BD4" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BE4" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BF4" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BG4" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BH4" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BI4" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BJ4" s="6" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="BK4" s="6" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="BL4" s="6" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="BM4" s="6" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="BN4" s="6" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="BO4" s="6" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="BP4" s="6" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="ET4" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="EU4" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="EV4" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1923,9 +1113,63 @@
           <t>L98</t>
         </is>
       </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="M5" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="N5" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Arregla el bug de actualizar info
</commit_message>
<xml_diff>
--- a/PlanStaffRGM.xlsx
+++ b/PlanStaffRGM.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Operations_best_opt" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operations_best_opt" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -15,8 +15,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -101,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -113,6 +114,7 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -478,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EX5"/>
+  <dimension ref="A1:GB8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -950,6 +952,96 @@
       <c r="EX1" s="1" t="n">
         <v>46041</v>
       </c>
+      <c r="EY1" s="11" t="n">
+        <v>46174</v>
+      </c>
+      <c r="EZ1" s="11" t="n">
+        <v>46175</v>
+      </c>
+      <c r="FA1" s="11" t="n">
+        <v>46176</v>
+      </c>
+      <c r="FB1" s="11" t="n">
+        <v>46177</v>
+      </c>
+      <c r="FC1" s="11" t="n">
+        <v>46178</v>
+      </c>
+      <c r="FD1" s="11" t="n">
+        <v>46179</v>
+      </c>
+      <c r="FE1" s="11" t="n">
+        <v>46180</v>
+      </c>
+      <c r="FF1" s="11" t="n">
+        <v>46181</v>
+      </c>
+      <c r="FG1" s="11" t="n">
+        <v>46182</v>
+      </c>
+      <c r="FH1" s="11" t="n">
+        <v>46183</v>
+      </c>
+      <c r="FI1" s="11" t="n">
+        <v>46184</v>
+      </c>
+      <c r="FJ1" s="11" t="n">
+        <v>46185</v>
+      </c>
+      <c r="FK1" s="11" t="n">
+        <v>46186</v>
+      </c>
+      <c r="FL1" s="11" t="n">
+        <v>46187</v>
+      </c>
+      <c r="FM1" s="11" t="n">
+        <v>46188</v>
+      </c>
+      <c r="FN1" s="11" t="n">
+        <v>46189</v>
+      </c>
+      <c r="FO1" s="11" t="n">
+        <v>46190</v>
+      </c>
+      <c r="FP1" s="11" t="n">
+        <v>46191</v>
+      </c>
+      <c r="FQ1" s="11" t="n">
+        <v>46192</v>
+      </c>
+      <c r="FR1" s="11" t="n">
+        <v>46193</v>
+      </c>
+      <c r="FS1" s="11" t="n">
+        <v>46194</v>
+      </c>
+      <c r="FT1" s="11" t="n">
+        <v>46195</v>
+      </c>
+      <c r="FU1" s="11" t="n">
+        <v>46196</v>
+      </c>
+      <c r="FV1" s="11" t="n">
+        <v>46197</v>
+      </c>
+      <c r="FW1" s="11" t="n">
+        <v>46198</v>
+      </c>
+      <c r="FX1" s="11" t="n">
+        <v>46199</v>
+      </c>
+      <c r="FY1" s="11" t="n">
+        <v>46200</v>
+      </c>
+      <c r="FZ1" s="11" t="n">
+        <v>46201</v>
+      </c>
+      <c r="GA1" s="11" t="n">
+        <v>46202</v>
+      </c>
+      <c r="GB1" s="11" t="n">
+        <v>46203</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1166,6 +1258,57 @@
       <c r="N5" s="5" t="inlineStr">
         <is>
           <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Data Analyst</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Vincent Rolong</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>L986</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Data Analyst</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Vincent Rolong</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>L989</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Supervisor</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Elver Gonzales</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>F69</t>
         </is>
       </c>
     </row>

</xml_diff>